<commit_message>
fix: format cell to text
</commit_message>
<xml_diff>
--- a/public/external_assessee.xlsx
+++ b/public/external_assessee.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adisa\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KPN Corp\KPN Assessment\kpn-assessment-fe\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AED623C6-FE62-40D0-87DE-CFAC4A8DB758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95FB8A3A-6DF1-4968-8C46-863A6BD7FF1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{AE52DA99-70B2-4F8F-B466-B27B534FADE6}"/>
+    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="7368" xr2:uid="{AE52DA99-70B2-4F8F-B466-B27B534FADE6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -110,13 +110,13 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -432,54 +432,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A50212E-EAFF-482F-984B-E9C9D019599B}">
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.21875" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="3"/>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B4" s="5"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="3"/>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B5" s="5"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -487,5 +475,6 @@
     <hyperlink ref="B3" r:id="rId2" xr:uid="{D8E4421C-B8C6-4DA3-90AA-C71F068CB4D2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix : xlsx upload assignee change
</commit_message>
<xml_diff>
--- a/public/external_assessee.xlsx
+++ b/public/external_assessee.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KPN Corp\KPN Assessment\kpn-assessment-fe\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95FB8A3A-6DF1-4968-8C46-863A6BD7FF1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="7368" xr2:uid="{AE52DA99-70B2-4F8F-B466-B27B534FADE6}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7320"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,30 +24,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>assessee_name</t>
   </si>
   <si>
     <t>assessee_email</t>
   </si>
-  <si>
-    <t>Jhon Doe</t>
-  </si>
-  <si>
-    <t>jhondoe@email.com</t>
-  </si>
-  <si>
-    <t>Jane Doe</t>
-  </si>
-  <si>
-    <t>janedoe@email.com</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -431,15 +418,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A50212E-EAFF-482F-984B-E9C9D019599B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.21875" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -447,34 +434,22 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>3</v>
-      </c>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+      <c r="B2" s="3"/>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>5</v>
-      </c>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="3"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" s="5"/>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" s="5"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{94867EF7-AC54-4E81-A119-6C495C4F8123}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{D8E4421C-B8C6-4DA3-90AA-C71F068CB4D2}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>